<commit_message>
Update on the tracking logic, so intermediate frames in an appearance can have facial landmarks. These frames are called waypoints.
</commit_message>
<xml_diff>
--- a/dataset_metadata.xlsx
+++ b/dataset_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uibes-my.sharepoint.com/personal/agc968_id_uib_eu/Documents/TFG/GEEIA-TFG-DFU/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marta\TFG\GEEIA-TFG-DFU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="247" documentId="8_{D3773089-7DAF-44F1-9F4B-4D9CCE4173E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FEF971DC-2B19-42A3-814F-864E411AEE19}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{092ADFCB-7F11-4E2B-A657-4238E16CF830}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2085" yWindow="4650" windowWidth="38700" windowHeight="15345" tabRatio="601" xr2:uid="{14AC8030-20A7-4C66-8027-B1BAD1A4B756}"/>
+    <workbookView xWindow="34290" yWindow="10440" windowWidth="17415" windowHeight="10545" tabRatio="601" xr2:uid="{14AC8030-20A7-4C66-8027-B1BAD1A4B756}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="129">
   <si>
     <t>p_0001_19052022_00.bag</t>
   </si>
@@ -389,12 +389,6 @@
     <t>[{"start_frame":937,"end_frame":991}]</t>
   </si>
   <si>
-    <t>[{"type":"PATIENT","appearances":[{"start":{"frame":153,"landmarks":{"left_eye":[580,384],"nose":[576,400],"mouth_left":[583,411]},"orientation":"TB"},"end":{"frame":164}},{"start":{"frame":381,"landmarks":{"left_eye":[851,158],"nose":[832,177],"mouth_left":[836,191]},"orientation":"TB"},"end":{"frame":393}},{"start":{"frame":394,"landmarks":{"left_eye":[838,122],"nose":[813,141],"mouth_left":[816,160]},"orientation":"TB"},"end":{"frame":398}},{"start":{"frame":399,"landmarks":{"left_eye":[836,87],"nose":[810,106],"mouth_left":[809,126]},"orientation":"TB"},"end":{"frame":402}},{"start":{"frame":403,"landmarks":{"left_eye":[843,45],"nose":[814,66],"mouth_left":[814,83]},"orientation":"TB"},"end":{"frame":434}}]}]</t>
-  </si>
-  <si>
-    <t>[{"type":"STAFF","appearances":[{"start":{"frame":115,"landmarks":{"mouth_right":[248,465],"mouth_left":[227,479]},"orientation":"BT"},"end":{"frame":229}},{"start":{"frame":257,"landmarks":{"mouth_right":[252,475]},"orientation":"BT"},"end":{"frame":281}}]},{"type":"PATIENT","appearances":[{"start":{"frame":794,"landmarks":{"mouth_right":[624,-3],"mouth_left":[643,6]},"orientation":"TB"},"end":{"frame":841}},{"start":{"frame":933,"landmarks":{"left_eye":[590,99]},"orientation":"TB"},"end":{"frame":940}}]}]</t>
-  </si>
-  <si>
     <t>[{"type":"PATIENT","appearances":[{"start":{"frame":126682,"landmarks":{"left_eye":[272,1]},"orientation":"TB"},"end":{"frame":126923}}]},{"type":"PATIENT","appearances":[{"start":{"frame":126913,"landmarks":{"right_eye":[1279,330]},"orientation":"TB"},"end":{"frame":127070}}]}]</t>
   </si>
   <si>
@@ -414,6 +408,21 @@
   </si>
   <si>
     <t>[{"type":"PATIENT","appearances":[{"start":{"frame":164689,"landmarks":{"right_eye":[151,330],"left_eye":[210,310]},"orientation":"TB"},"end":{"frame":165242}}]},{"type":"UNKNOWN","appearances":[{"start":{"frame":165056,"landmarks":{"right_eye":[-2,101],"left_eye":[9,97],"nose":[6,108]},"orientation":"TB"},"end":{"frame":165078}},{"start":{"frame":165106,"landmarks":{"right_eye":[35,145],"left_eye":[47,141]},"orientation":"TB"},"end":{"frame":165169}}]},{"type":"STAFF","appearances":[{"start":{"frame":164689,"landmarks":{"right_eye":[126,182],"left_eye":[150,169],"nose":[146,190],"mouth_right":[144,205],"mouth_left":[163,197]},"orientation":"TB"},"end":{"frame":164755}},{"start":{"frame":165001,"landmarks":{"nose":[256,0],"mouth_right":[266,10],"mouth_left":[275,-1]},"orientation":"TB"},"end":{"frame":165012}}]}]</t>
+  </si>
+  <si>
+    <t>[{"type":"STAFF","appearances":[{"start":{"frame":80,"landmarks":{"left_eye":[-4,444],"right_eye":[4,381]},"orientation":"RL"},"end":{"frame":122}}]},{"type":"PATIENT","appearances":[{"start":{"frame":148,"landmarks":{"left_eye":[564,404],"nose":[560,421],"mouth_left":[570,432]},"orientation":"TB"},"waypoints":[{"frame":153,"landmarks":{"left_eye":[580,384],"nose":[575,400],"mouth_left":[583,411]},"orientation":"TB"}],"end":{"frame":165}},{"start":{"frame":381,"landmarks":{"left_eye":[851,158],"nose":[832,177],"mouth_left":[836,191]},"orientation":"TB"},"waypoints":[{"frame":394,"landmarks":{"left_eye":[838,122],"nose":[813,141],"mouth_left":[816,160]},"orientation":"TB"},{"frame":399,"landmarks":{"left_eye":[836,87],"nose":[810,106],"mouth_left":[809,126]},"orientation":"TB"},{"frame":403,"landmarks":{"left_eye":[843,45],"nose":[814,66],"mouth_left":[814,83]},"orientation":"TB"}],"end":{"frame":433}}]}]</t>
+  </si>
+  <si>
+    <t>[{"type":"STAFF","appearances":[{"start":{"frame":115,"landmarks":{"mouth_right":[248,465],"mouth_left":[227,479]},"orientation":"BT"},"end":{"frame":229}},{"start":{"frame":257,"landmarks":{"mouth_right":[252,475]},"orientation":"BT"},"end":{"frame":281}},{"start":{"frame":1158,"landmarks":{"right_eye":[593,294],"left_eye":[591,332],"nose":[560,306],"mouth_right":[553,293],"mouth_left":[551,318]},"orientation":"RL"},"end":{"frame":1196}}]},{"type":"PATIENT","appearances":[{"start":{"frame":794,"landmarks":{"mouth_right":[624,-3],"mouth_left":[643,6]},"orientation":"TB"},"end":{"frame":841}},{"start":{"frame":933,"landmarks":{"left_eye":[590,99]},"orientation":"TB"},"end":{"frame":940}}]}]</t>
+  </si>
+  <si>
+    <t>[{"start_frame":42,"end_frame":94},{"start_frame":239,"end_frame":270},{"start_frame":1012,"end_frame":1090}]</t>
+  </si>
+  <si>
+    <t>[{"start_frame":95,"end_frame":121},{"start_frame":136,"end_frame":153},{"start_frame":157,"end_frame":182},{"start_frame":188,"end_frame":227},{"start_frame":232,"end_frame":238},{"start_frame":271,"end_frame":321},{"start_frame":326,"end_frame":348},{"start_frame":364,"end_frame":372},{"start_frame":376,"end_frame":433},{"start_frame":450,"end_frame":512},{"start_frame":517,"end_frame":549},{"start_frame":553,"end_frame":620}]</t>
+  </si>
+  <si>
+    <t>[{"type":"PATIENT","appearances":[{"start":{"frame":724,"landmarks":{"left_eye":[0,151]},"orientation":"TB"},"waypoints":[{"frame":726,"landmarks":{"left_eye":[15,152],"mouth_left":[0,173]},"orientation":"TB"},{"frame":728,"landmarks":{"left_eye":[21,148],"nose":[-1,138],"mouth_left":[7,167]},"orientation":"TB"},{"frame":925,"landmarks":{"right_eye":[129,223],"left_eye":[154,228],"nose":[137,224],"mouth_right":[122,238],"mouth_left":[140,244]},"orientation":"TB"},{"frame":927,"landmarks":{"right_eye":[131,192],"left_eye":[155,198],"nose":[140,196],"mouth_right":[126,210],"mouth_left":[143,215]},"orientation":"TB"},{"frame":929,"landmarks":{"right_eye":[127,157],"left_eye":[151,163],"nose":[137,160],"mouth_right":[120,175],"mouth_left":[141,184]},"orientation":"TB"},{"frame":931,"landmarks":{"right_eye":[123,118],"left_eye":[149,126],"nose":[133,121],"mouth_right":[117,134],"mouth_left":[139,143]},"orientation":"TB"},{"frame":933,"landmarks":{"right_eye":[115,78],"left_eye":[142,84],"nose":[127,80],"mouth_right":[111,92],"mouth_left":[131,99]},"orientation":"TB"},{"frame":935,"landmarks":{"right_eye":[102,28],"left_eye":[129,37],"nose":[116,31],"mouth_right":[97,41],"mouth_left":[121,52]},"orientation":"TB"}],"end":{"frame":937}}]},{"type":"STAFF","appearances":[{"start":{"frame":771,"landmarks":{"left_eye":[0,182]},"orientation":"TB"},"waypoints":[{"frame":775,"landmarks":{"left_eye":[12,188],"mouth_left":[0,203]},"orientation":"TB"},{"frame":777,"landmarks":{"right_eye":[-1,184],"left_eye":[18,192],"nose":[1,193],"mouth_left":[5,206]},"orientation":"TB"}],"end":{"frame":815}}]}]</t>
   </si>
 </sst>
 </file>
@@ -832,10 +841,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1380,7 +1385,7 @@
         <v>85</v>
       </c>
       <c r="M7" s="37" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="13.5" x14ac:dyDescent="0.25">
@@ -1411,7 +1416,7 @@
       <c r="K8" s="33"/>
       <c r="L8" s="33"/>
       <c r="M8" s="40" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="13.5" x14ac:dyDescent="0.25">
@@ -1616,7 +1621,7 @@
       <c r="K15" s="14"/>
       <c r="L15" s="14"/>
       <c r="M15" s="36" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="13.5" x14ac:dyDescent="0.25">
@@ -1851,7 +1856,7 @@
       <c r="K24" s="20"/>
       <c r="L24" s="20"/>
       <c r="M24" s="52" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="N24" s="4"/>
     </row>
@@ -2054,7 +2059,7 @@
       <c r="K32" s="20"/>
       <c r="L32" s="20"/>
       <c r="M32" s="52" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="N32" s="4"/>
     </row>
@@ -2268,7 +2273,7 @@
       <c r="K41" s="14"/>
       <c r="L41" s="14"/>
       <c r="M41" s="36" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="N41" s="4"/>
     </row>
@@ -2828,7 +2833,7 @@
       <c r="K65" s="14"/>
       <c r="L65" s="14"/>
       <c r="M65" s="36" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="N65" s="4"/>
     </row>
@@ -2960,14 +2965,24 @@
       <c r="E71" s="61" t="s">
         <v>69</v>
       </c>
-      <c r="F71" s="11"/>
-      <c r="G71" s="11"/>
+      <c r="F71" s="11">
+        <v>42</v>
+      </c>
+      <c r="G71" s="11">
+        <v>1090</v>
+      </c>
       <c r="H71" s="12"/>
-      <c r="I71" s="13"/>
-      <c r="J71" s="14"/>
+      <c r="I71" s="61" t="s">
+        <v>126</v>
+      </c>
+      <c r="J71" s="36" t="s">
+        <v>127</v>
+      </c>
       <c r="K71" s="14"/>
       <c r="L71" s="14"/>
-      <c r="M71" s="14"/>
+      <c r="M71" s="36" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="72" spans="1:14" ht="13.5" x14ac:dyDescent="0.25">
       <c r="A72" s="38">
@@ -3035,7 +3050,7 @@
       <c r="K74" s="20"/>
       <c r="L74" s="20"/>
       <c r="M74" s="52" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
     </row>
     <row r="75" spans="1:14" ht="13.5" x14ac:dyDescent="0.25">
@@ -3070,7 +3085,7 @@
         <v>91</v>
       </c>
       <c r="M75" s="53" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -3081,15 +3096,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101000620FAD95693C64EA031EEF30A884E22" ma:contentTypeVersion="18" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="3cb1aab9e578f80d2fc4686fbfe751cf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="fafbbf91-3bff-4810-9140-1154e687d00d" xmlns:ns4="b6e30ae0-770c-4ded-9a45-db310f4376cf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dd71c47001de44f1b40c6be5bf6ee2fe" ns3:_="" ns4:_="">
     <xsd:import namespace="fafbbf91-3bff-4810-9140-1154e687d00d"/>
@@ -3342,7 +3348,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_activity xmlns="b6e30ae0-770c-4ded-9a45-db310f4376cf" xsi:nil="true"/>
@@ -3350,15 +3356,16 @@
 </p:properties>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EBFD5DB7-20B3-4413-B343-207357287550}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A7A7063-C8C0-4D53-85FB-FA1C7D034925}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3377,7 +3384,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54E07BE4-568A-4A33-A47A-9A6DE9B672F8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
@@ -3392,4 +3399,12 @@
     <ds:schemaRef ds:uri="b6e30ae0-770c-4ded-9a45-db310f4376cf"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EBFD5DB7-20B3-4413-B343-207357287550}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>